<commit_message>
QA 2026-10-17: LP·연동 success, GP success
</commit_message>
<xml_diff>
--- a/2026-10-17/2026-10-17-gp.xlsx
+++ b/2026-10-17/2026-10-17-gp.xlsx
@@ -47,7 +47,7 @@
     <t>실행 시각 (KST)</t>
   </si>
   <si>
-    <t>2026-10-17 02:43</t>
+    <t>2026-10-17 04:21</t>
   </si>
   <si>
     <t>환경</t>
@@ -59,7 +59,7 @@
     <t>코드 버전</t>
   </si>
   <si>
-    <t>LP 7f010fa · GP 3315740</t>
+    <t>LP fd9a067 · GP a45c340</t>
   </si>
   <si>
     <t>데이터</t>

</xml_diff>